<commit_message>
feat: retry transient API errors, 7 sample clients, shorter README
- one retry with backoff for timeouts, 429 and 5xx; 401/402/403 fail fast
- tests for retry logic with a fake OpenAI client (30 tests)
- journal stores PDF/TXT paths relative to output folder
- ProxyAPI defaults per docs: https://api.proxyapi.ru/v1 + openai/gpt-5-mini
- macOS Arial font fallback; README quick start for Windows and macOS/Linux
- refresh live-check: endpoint reachable, current key rejected (HTTP 401)
</commit_message>
<xml_diff>
--- a/examples/clients.xlsx
+++ b/examples/clients.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,12 +458,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Анна</t>
+          <t>Анна Соколова</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Telegram-бот для предзаказа кофе с меню и уведомлением сотрудника о новом заказе</t>
+          <t>Telegram-бот для предзаказа кофе: меню с ценами, выбор времени получения, уведомление бариста о новом заказе</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -473,17 +473,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Студия Линия</t>
+          <t>Студия дизайна Линия</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Михаил</t>
+          <t>Михаил Орлов</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Сайт с портфолио дизайнера и формой заявки на консультацию</t>
+          <t>Сайт-портфолио дизайнера интерьеров с галереей проектов и формой записи на консультацию</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -493,21 +493,101 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Сервис Вектор</t>
+          <t>Логистика Вектор</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Елена</t>
+          <t>Елена Кравцова</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Автоматизация сбора заявок из таблицы и подготовки ежедневного отчёта менеджеру</t>
+          <t>Автоматический сбор заявок из Google-таблицы и ежедневный отчёт руководителю отдела продаж на почту</t>
         </is>
       </c>
       <c r="D4" t="n">
         <v>60000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Стоматология Улыбка Плюс</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ирина Белова</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Онлайн-запись пациентов к врачам с SMS-напоминанием за сутки и учётом свободных окон в расписании</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Автосервис ГаражПро</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Дмитрий Захаров</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Чат-бот в WhatsApp для приёма заявок на ремонт, предварительной оценки стоимости по типу работ и записи на время</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>95000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Интернет-магазин ЭкоДом</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ольга Миронова</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Интеграция магазина на Tilda с CRM: передача заказов, статусы доставки и автоматические письма покупателям</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>220000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Школа английского Talk Up</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Сергей Ветров</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Личный кабинет ученика с расписанием занятий, домашними заданиями и напоминаниями в Telegram</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>350000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>